<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.003-06 L'abeille en bois du marché
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.003-06.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.003-06.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>L'abeille cachée et le miel</t>
+          <t>L'abeille en bois du marché</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>marché, stand de paille puis miel</t>
+          <t>marché, pots dorés, stand des pots, panier de rotin, pain, prunes, muret</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nina, Aniss, maman</t>
+          <t>Nina, Aniss, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut montrer l'abeille en bois à Aniss, puis un pot de miel pour le pain du soir. L'abeille est cachée. Aniss la voit. Le miel rentre dans le sac.</t>
+          <t>Un rayon allume le bord du panier. Au bord, un éclat de rotin brille. Nina veut montrer l'abeille en bois, maintenant. Aniss arrive. Un rire commence. Aniss se tait. Un pot tape. Nina refuse de foncer. Ils regardent derrière, à deux. Merci vécu. Le pot glisse. L'éclat de rotin tient au bord.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une poule picore près des caisses de paille. Elle fait un petit cot-cot. Une plume grise tourne au sol. Ça sent le grain et le bois. Maman tient le panier de rotin. Le rotin est rêche et chaud. Un rayon passe entre les toiles. Tu as vu la plume, Nina ? Elle tourne. Oui. La poule l'a laissée. Nina ramasse la plume. Elle est légère et douce. Je la pose là. Près du panier. En ce moment, Nina cherche l'abeille. Les pots dorés brillent un peu. L'abeille en bois. Je veux la montrer. Elle est au stand de miel. Collée sur la caisse. Aniss arrive près des pots. Aniss a des lunettes neuves. Aniss a les cheveux courts. Il porte un gilet bleu. Aniss, tu regardes avec Nina. Tu viens voir l'abeille ? Oui. Les pots dorés sont serrés. Ça sent le sucré et la cire. L'abeille n'est pas devant. Elle n'est plus là. On peut regarder derrière. Tout doux, sans bouger les pots. Aniss se penche. Il voit les ailes peintes. Derrière le gros pot. Elle est collée.</t>
+          <t>Un rayon glisse entre les toiles du marché. Il allume le bord du panier. Tu le vois, Nina ? Oui, ça brille. Papa tient le panier de rotin. Le rotin est rêche, un peu chaud. Au bord, un éclat de rotin brille. Il pique un peu, papa. Tu le sens, sous le doigt ? Oui, un petit point. Le panier sent le pain, Nina ? Un peu, maman. Le pain chaud tape le bras de maman. Il est tiède. On le pose près des pots ? Oui. Les pots dorés brillent, serrés. L'abeille en bois, maman. Je veux la montrer, maintenant ! Elle est au stand des pots ? Oui, collée derrière. Tu la cherches, Nina ? Oui, papa. En ce moment, Nina cherche l'abeille. Les pots sentent le sucré, un peu la cire. Elle n'est pas devant. On avance sans bousculer ? Oui. Aniss arrive près des pots. Ses chaussures font un petit bruit. Aniss a des lunettes. Aniss a les cheveux courts. Il porte un gilet bleu. Aniss, tu regardes avec Nina ? Oui. Tu viens voir l'abeille ? Oui. Nina regarde les lunettes, trop longtemps. Un rire commence dans sa bouche. Aniss ne dit rien. Le sourire d'Aniss disparaît. Tu te penches, maintenant ! Non. Oh. Nina avance trop vite vers les pots. Un pot tape un autre, sec. Ça fait un bruit dur. Elle n'est plus là ! Elle est cachée. L'éclat de rotin tremble, puis tient. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Nina ? Oui, papa. Tes mains sont collantes, Nina ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une poule picore près des caisses de paille. Elle fait un petit cot-cot. Une plume grise tourne au sol. Ça sent le grain et le bois. Maman tient le panier de rotin. Le rotin est rêche et chaud. Un rayon passe entre les toiles. Tu as vu la plume, Nina ? Elle tourne. Oui. La poule l'a laissée. Nina ramasse la plume. Elle est légère et douce. Je la pose là. Près du panier. En ce moment, Nina cherche l'abeille. Les pots dorés brillent un peu. L'abeille en bois. Je veux la montrer. Elle est au stand de miel. Collée sur la caisse. Aniss arrive près des pots. Aniss a des lunettes neuves. Aniss a les cheveux courts. Il porte un gilet bleu. Aniss, tu regardes avec Nina. Tu viens voir l'abeille ? Oui. Les pots dorés sont serrés. Ça sent le sucré et la cire. L'abeille n'est pas devant. Elle n'est plus là. On peut regarder derrière. Tout doux, sans bouger les pots. Aniss se penche. Il voit les ailes peintes. Derrière le gros pot. Elle est collée.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un rayon glisse entre les toiles du marché. Il allume le bord du panier. Tu le vois, Nina ? Oui, ça brille. Papa tient le panier de rotin. Le rotin est rêche, un peu chaud. Au bord, un &lt;emphasis level="moderate"&gt;éclat de rotin&lt;/emphasis&gt; brille. Il pique un peu, papa. Tu le sens, sous le doigt ? Oui, un petit point. Le panier sent le pain, Nina ? Un peu, maman. Le pain chaud tape le bras de maman. Il est tiède. On le pose près des pots ? Oui. Les pots dorés brillent, serrés. L'abeille en bois, maman. Je veux la montrer, maintenant ! Elle est au stand des pots ? Oui, collée derrière. Tu la cherches, Nina ? Oui, papa. En ce moment, Nina cherche l'abeille. Les pots sentent le sucré, un peu la cire. Elle n'est pas devant. On avance sans bousculer ? Oui. Aniss arrive près des pots. Ses chaussures font un petit bruit. Aniss a des lunettes. Aniss a les cheveux courts. Il porte un gilet bleu. Aniss, tu regardes avec Nina ? Oui. Tu viens voir l'abeille ? Oui. Nina regarde les lunettes, trop longtemps. Un rire commence dans sa bouche. Aniss ne dit rien. Le sourire d'Aniss disparaît. Tu te penches, maintenant ! Non. Oh. Nina avance trop vite vers les pots. Un pot tape un autre, sec. Ça fait un bruit dur. Elle n'est plus là ! Elle est cachée. L'éclat de rotin tremble, puis tient. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Nina ? Oui, papa. Tes mains sont collantes, Nina ? Un peu, maman.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Agathe est au marché avec maman. Barnabé arrive avec des lunettes neuves. Un camarade ouvre la bouche. Agathe ne rit &lt;emphasis&gt;pas&lt;/emphasis&gt;. Il ne faut pas rire de l'apparence. Maman dit : on joue. On ne rit pas des lunettes, des cheveux ou d'un habit. Agathe tend une prune. Elles marchent ensemble. Pas rire de l'apparence. [pause]</t>
+          <t>Un rayon glisse entre les toiles du marché. Il allume le bord du panier. Tu le vois, Nina ? Oui, ça brille. Papa tient le panier de rotin. Le rotin est rêche, un peu chaud. Au bord, un &lt;emphasis&gt;éclat de rotin&lt;/emphasis&gt; brille. Il pique un peu, papa. Tu le sens, sous le doigt ? Oui, un petit point. Le panier sent le pain, Nina ? Un peu, maman. Le pain chaud tape le bras de maman. Il est tiède. On le pose près des pots ? Oui. Les pots dorés brillent, serrés. L'abeille en bois, maman. Je veux la montrer, maintenant ! Elle est au stand des pots ? Oui, collée derrière. Tu la cherches, Nina ? Oui, papa. En ce moment, Nina cherche l'abeille. Les pots sentent le sucré, un peu la cire. Elle n'est pas devant. On avance sans bousculer ? Oui. Aniss arrive près des pots. Ses chaussures font un petit bruit. Aniss a des lunettes. Aniss a les cheveux courts. Il porte un gilet bleu. Aniss, tu regardes avec Nina ? Oui. Tu viens voir l'abeille ? Oui. Nina regarde les lunettes, trop longtemps. Un rire commence dans sa bouche. Aniss ne dit rien. Le sourire d'Aniss disparaît. Tu te penches, maintenant ! Non. Oh. Nina avance trop vite vers les pots. Un pot tape un autre, sec. Ça fait un bruit dur. Elle n'est plus là ! Elle est cachée. L'éclat de rotin tremble, puis tient. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Nina ? Oui, papa. Tes mains sont collantes, Nina ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>éclat de rotin</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,52 +1321,76 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_montrer_l_abeille_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une poule picore près des caisses de paille.
-narrateur|Elle fait un petit cot-cot.
-narrateur|Une plume grise tourne au sol.
-narrateur|Ça sent le grain et le bois.
-narrateur|Maman tient le panier de rotin.
-narrateur|Le rotin est rêche et chaud.
-narrateur|Un rayon passe entre les toiles.
-maman|Tu as vu la plume, Nina ?
-enfant-f|Elle tourne.
-maman|Oui.
-maman|La poule l'a laissée.
-narrateur|Nina ramasse la plume.
-narrateur|Elle est légère et douce.
-enfant-f|Je la pose là.
-maman|Près du panier.
+          <t>narrateur|Un rayon glisse entre les toiles du marché.
+narrateur|Il allume le bord du panier.
+papa|Tu le vois, Nina ?
+enfant-f|Oui, ça brille.
+narrateur|Papa tient le panier de rotin.
+narrateur|Le rotin est rêche, un peu chaud.
+narrateur|Au bord, un éclat de rotin brille.
+enfant-f|Il pique un peu, papa.
+papa|Tu le sens, sous le doigt ?
+enfant-f|Oui, un petit point.
+maman|Le panier sent le pain, Nina ?
+enfant-f|Un peu, maman.
+narrateur|Le pain chaud tape le bras de maman.
+enfant-f|Il est tiède.
+maman|On le pose près des pots ?
+enfant-f|Oui.
+narrateur|Les pots dorés brillent, serrés.
+enfant-f|L'abeille en bois, maman.
+enfant-f|Je veux la montrer, maintenant !
+maman|Elle est au stand des pots ?
+enfant-f|Oui, collée derrière.
+papa|Tu la cherches, Nina ?
+enfant-f|Oui, papa.
 narrateur|En ce moment, Nina cherche l'abeille.
-narrateur|Les pots dorés brillent un peu.
-enfant-f|L'abeille en bois.
-enfant-f|Je veux la montrer.
-maman|Elle est au stand de miel.
-maman|Collée sur la caisse.
+narrateur|Les pots sentent le sucré, un peu la cire.
+enfant-f|Elle n'est pas devant.
+maman|On avance sans bousculer ?
+enfant-f|Oui.
 narrateur|Aniss arrive près des pots.
-narrateur|Aniss a des lunettes neuves.
+narrateur|Ses chaussures font un petit bruit.
+narrateur|Aniss a des lunettes.
 narrateur|Aniss a les cheveux courts.
 narrateur|Il porte un gilet bleu.
-maman|Aniss, tu regardes avec Nina.
+papa|Aniss, tu regardes avec Nina ?
+copain|Oui.
 enfant-f|Tu viens voir l'abeille ?
 copain|Oui.
-narrateur|Les pots dorés sont serrés.
-narrateur|Ça sent le sucré et la cire.
-narrateur|L'abeille n'est pas devant.
-enfant-f|Elle n'est plus là.
-maman|On peut regarder derrière.
-maman|Tout doux, sans bouger les pots.
-narrateur|Aniss se penche.
-narrateur|Il voit les ailes peintes.
-copain|Derrière le gros pot.
-copain|Elle est collée.</t>
+narrateur|Nina regarde les lunettes, trop longtemps.
+narrateur|Un rire commence dans sa bouche.
+narrateur|Aniss ne dit rien.
+narrateur|Le sourire d'Aniss disparaît.
+enfant-f|Tu te penches, maintenant !
+copain|Non.
+enfant-f|Oh.
+narrateur|Nina avance trop vite vers les pots.
+narrateur|Un pot tape un autre, sec.
+narrateur|Ça fait un bruit dur.
+enfant-f|Elle n'est plus là !
+copain|Elle est cachée.
+narrateur|L'éclat de rotin tremble, puis tient.
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Aniss, Nina ?
+enfant-f|Oui, papa.
+maman|Tes mains sont collantes, Nina ?
+enfant-f|Un peu, maman.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>marche,miel</t>
+          <t>marche</t>
         </is>
       </c>
     </row>
@@ -1398,22 +1422,22 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aniss a des lunettes. Que fait Nina ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Aniss a des &lt;emphasis level="moderate"&gt;lunettes&lt;/emphasis&gt;. Que fait Nina ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Barnabé a des lunettes. Que fait Agathe ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Aniss a des &lt;emphasis&gt;lunettes&lt;/emphasis&gt;. Que fait Nina ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>jouer</t>
+          <t>pas rire</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>jouer | ensemble | montrer | abeille | on joue | pas rire</t>
+          <t>pas rire | jouer | ensemble</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1428,7 +1452,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Nina montre l'abeille. Que fait-elle ?</t>
+          <t>Nina montre l'abeille. Que fait Nina ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1466,7 +1490,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1477,7 +1501,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1492,34 +1516,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>lunettes</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1534,17 +1562,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=aniss_a_des_lunettes_nina_ne_rit_pas; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1577,17 +1605,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina se penche aussi. L'abeille en bois est là. Elle a des ailes peintes. Jaune. Et noire. Merci, Nina. Merci, Aniss. Aniss a vu derrière. L'abeille est là. On prend du miel ? Un petit pot. Pour le pain du soir. Maman choisit un pot doré. Le couvercle est un peu collant. Ça sent le sucré. C'est épais. Oui. C'est le miel.</t>
+          <t>Nina veut l'abeille, tout de suite. Je me penche, maintenant ! Elle avance trop vite vers Aniss. Les mots se bousculent dans sa bouche. Non. Aniss reste un peu plus loin. Oh. Le sourire ne revient pas. Nina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe les pots, un instant. Elle écoute le rotin du panier. Tu veux l'abeille avec Aniss ? Papa reste à la même hauteur. Tu regardes derrière ? Aniss ne dit rien, d'abord. Il se penche près du gros pot. Je vois les ailes. D'accord. Merci, Nina. Papa a vu les deux, près des pots. Le pot est collant, sous les doigts. Il sent le sucré. Ils regardent derrière, sans se presser. Aniss montre les ailes peintes. Là. Je la vois. Jaune. Et noire. Tu la vois, l'abeille ? Oui, papa. Un petit pot, Nina ? Pour le pain du soir. Maman choisit un pot doré. Nina tient le bord, plus près. Il est lourd. Oui. Le ventre de Nina se desserre. Les épaules se relèvent un peu. On reste près des pots ? Oui. Tes mains sont au chaud ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina se penche aussi. L'abeille en bois est là. Elle a des ailes peintes. Jaune. Et noire. Merci, Nina. Merci, Aniss. Aniss a vu derrière. L'abeille est là. On prend du miel ? Un petit pot. Pour le pain du soir. Maman choisit un pot doré. Le couvercle est un peu collant. Ça sent le sucré. C'est épais. Oui. C'est le miel.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina veut l'&lt;emphasis level="moderate"&gt;abeille&lt;/emphasis&gt;, tout de suite. Je me penche, maintenant ! Elle avance trop vite vers Aniss. Les mots se bousculent dans sa bouche. Non. Aniss reste un peu plus loin. Oh. Le sourire ne revient pas. Nina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe les pots, un instant. Elle écoute le rotin du panier. Tu veux l'abeille avec Aniss ? Papa reste à la même hauteur. Tu regardes derrière ? Aniss ne dit rien, d'abord. Il se penche près du gros pot. Je vois les ailes. D'accord. Merci, Nina. Papa a vu les deux, près des pots. Le pot est collant, sous les doigts. Il sent le sucré. Ils regardent derrière, sans se presser. Aniss montre les ailes peintes. Là. Je la vois. Jaune. Et noire. Tu la vois, l'abeille ? Oui, papa. Un petit pot, Nina ? Pour le pain du soir. Maman choisit un pot doré. Nina tient le bord, plus près. Il est lourd. Oui. Le ventre de Nina se desserre. Les épaules se relèvent un peu. On reste près des pots ? Oui. Tes mains sont au chaud ? Un peu, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Agathe n'a &lt;emphasis&gt;pas&lt;/emphasis&gt; ri. Elle a joué. Pas rire de l'apparence. [pause]</t>
+          <t>Nina veut l'&lt;emphasis&gt;abeille&lt;/emphasis&gt;, tout de suite. Je me penche, maintenant ! Elle avance trop vite vers Aniss. Les mots se bousculent dans sa bouche. Non. Aniss reste un peu plus loin. Oh. Le sourire ne revient pas. Nina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe les pots, un instant. Elle écoute le rotin du panier. Tu veux l'abeille avec Aniss ? Papa reste à la même hauteur. Tu regardes derrière ? Aniss ne dit rien, d'abord. Il se penche près du gros pot. Je vois les ailes. D'accord. Merci, Nina. Papa a vu les deux, près des pots. Le pot est collant, sous les doigts. Il sent le sucré. Ils regardent derrière, sans se presser. Aniss montre les ailes peintes. Là. Je la vois. Jaune. Et noire. Tu la vois, l'abeille ? Oui, papa. Un petit pot, Nina ? Pour le pain du soir. Maman choisit un pot doré. Nina tient le bord, plus près. Il est lourd. Oui. Le ventre de Nina se desserre. Les épaules se relèvent un peu. On reste près des pots ? Oui. Tes mains sont au chaud ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1634,7 +1662,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1642,10 +1670,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1668,30 +1696,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>abeille</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1700,10 +1728,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1716,29 +1744,60 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=ils_regardent_derriere_a_deux; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina se penche aussi.
-narrateur|L'abeille en bois est là.
-narrateur|Elle a des ailes peintes.
+          <t>narrateur|Nina veut l'abeille, tout de suite.
+enfant-f|Je me penche, maintenant !
+narrateur|Elle avance trop vite vers Aniss.
+narrateur|Les mots se bousculent dans sa bouche.
+copain|Non.
+narrateur|Aniss reste un peu plus loin.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Nina refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe les pots, un instant.
+narrateur|Elle écoute le rotin du panier.
+papa|Tu veux l'abeille avec Aniss ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|Tu regardes derrière ?
+narrateur|Aniss ne dit rien, d'abord.
+narrateur|Il se penche près du gros pot.
+copain|Je vois les ailes.
+enfant-f|D'accord.
+papa|Merci, Nina.
+narrateur|Papa a vu les deux, près des pots.
+maman|Le pot est collant, sous les doigts.
+enfant-f|Il sent le sucré.
+narrateur|Ils regardent derrière, sans se presser.
+narrateur|Aniss montre les ailes peintes.
+copain|Là.
+enfant-f|Je la vois.
 enfant-f|Jaune.
 copain|Et noire.
-maman|Merci, Nina.
-maman|Merci, Aniss.
-maman|Aniss a vu derrière.
-maman|L'abeille est là.
-enfant-f|On prend du miel ?
-maman|Un petit pot.
-maman|Pour le pain du soir.
+papa|Tu la vois, l'abeille ?
+enfant-f|Oui, papa.
+maman|Un petit pot, Nina ?
+enfant-f|Pour le pain du soir.
 narrateur|Maman choisit un pot doré.
-narrateur|Le couvercle est un peu collant.
-enfant-f|Ça sent le sucré.
-copain|C'est épais.
-maman|Oui.
-maman|C'est le miel.</t>
+narrateur|Nina tient le bord, plus près.
+enfant-f|Il est lourd.
+copain|Oui.
+narrateur|Le ventre de Nina se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près des pots ?
+enfant-f|Oui.
+maman|Tes mains sont au chaud ?
+enfant-f|Un peu, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>pots</t>
         </is>
       </c>
     </row>
@@ -1765,17 +1824,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Le pot glisse dans le panier. Le rotin crisse. Vous voulez une prune ? Oui. Nina tend une prune à Aniss. La prune est lisse et froide. Merci. Ils croquent près du muret. Le muret est un peu rêche. Le jus est sucré. Bravo. Tu as montré l'abeille. On peut la revoir ? Un dernier regard. L'abeille brille encore. La poule picore plus loin. La plume ne tourne plus. Ce soir, le pain et le miel. Oui. Avec le petit pot. Sur le pain chaud. Le panier sent déjà le sucré.</t>
+          <t>Nina veut prendre le pot, trop vite. Je le mets, d'un coup ! Le pot glisse vers le bord. Ça tombe ! Attends. Aniss recule d'un pas. Nina avance les mains, trop vite. Elle regarde les lunettes, trop longtemps. Un rire revient dans sa bouche. Non. Oh. Le pot penche, collant. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe l'abeille, un instant. Elle écoute le rotin du panier. Au bord, un éclat de rotin luit. Là, sur le bord. Tu tiens avec moi ? Aniss ne dit rien. Il pose les mains sur le pot. Oui. Ils posent le pot, sans se presser. L'abeille en bois reste collée. Elle est là. Derrière. Tu l'as montrée, Nina ? Oui, papa. Le gilet est chaud, Aniss ? Un peu. Le pot glisse dans le panier. On passe près du muret ? J'y vais. Nina marche à côté d'Aniss. Le gilet bleu bouge. Les lunettes restent sur le nez. C'est plus facile. Le panier est lourd ? Un peu, papa. Un rayon passe entre les toiles. Il allume le pot. Ils passent près des prunes. Elles sont lisses. On va jusqu'au muret ? Oui, maman.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Le pot glisse dans le panier. Le rotin crisse. Vous voulez une prune ? Oui. Nina tend une prune à Aniss. La prune est lisse et froide. Merci. Ils croquent près du muret. Le muret est un peu rêche. Le jus est sucré. Bravo. Tu as montré l'abeille. On peut la revoir ? Un dernier regard. L'abeille brille encore. La poule picore plus loin. La plume ne tourne plus. Ce soir, le pain et le miel. Oui. Avec le petit pot. Sur le pain chaud. Le panier sent déjà le sucré.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina veut prendre le pot, trop vite. Je le mets, d'un coup ! Le pot glisse vers le bord. Ça tombe ! Attends. Aniss recule d'un pas. Nina avance les mains, trop vite. Elle regarde les lunettes, trop longtemps. Un rire revient dans sa bouche. Non. Oh. Le pot penche, collant. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe l'abeille, un instant. Elle écoute le rotin du panier. Au bord, un &lt;emphasis level="moderate"&gt;éclat de rotin&lt;/emphasis&gt; luit. Là, sur le bord. Tu tiens avec moi ? Aniss ne dit rien. Il pose les mains sur le pot. Oui. Ils posent le pot, sans se presser. L'abeille en bois reste collée. Elle est là. Derrière. Tu l'as montrée, Nina ? Oui, papa. Le gilet est chaud, Aniss ? Un peu. Le pot glisse dans le panier. On passe près du muret ? J'y vais. Nina marche à côté d'Aniss. Le gilet bleu bouge. Les lunettes restent sur le nez. C'est plus facile. Le panier est lourd ? Un peu, papa. Un rayon passe entre les toiles. Il allume le pot. Ils passent près des prunes. Elles sont lisses. On va jusqu'au muret ? Oui, maman.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman achète du pain. Agathe donne la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Nina veut prendre le pot, trop vite. Je le mets, d'un coup ! Le pot glisse vers le bord. Ça tombe ! Attends. Aniss recule d'un pas. Nina avance les mains, trop vite. Elle regarde les lunettes, trop longtemps. Un rire revient dans sa bouche. Non. Oh. Le pot penche, collant. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe l'abeille, un instant. Elle écoute le rotin du panier. Au bord, un &lt;emphasis&gt;éclat de rotin&lt;/emphasis&gt; luit. Là, sur le bord. Tu tiens avec moi ? Aniss ne dit rien. Il pose les mains sur le pot. Oui. Ils posent le pot, sans se presser. L'abeille en bois reste collée. Elle est là. Derrière. Tu l'as montrée, Nina ? Oui, papa. Le gilet est chaud, Aniss ? Un peu. Le pot glisse dans le panier. On passe près du muret ? J'y vais. Nina marche à côté d'Aniss. Le gilet bleu bouge. Les lunettes restent sur le nez. C'est plus facile. Le panier est lourd ? Un peu, papa. Un rayon passe entre les toiles. Il allume le pot. Ils passent près des prunes. Elles sont lisses. On va jusqu'au muret ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1822,7 +1881,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1830,10 +1889,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1856,30 +1915,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de rotin</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1888,10 +1947,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1902,31 +1961,64 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Le pot glisse dans le panier.
-narrateur|Le rotin crisse.
-maman|Vous voulez une prune ?
-enfant-f|Oui.
-narrateur|Nina tend une prune à Aniss.
-narrateur|La prune est lisse et froide.
-copain|Merci.
-narrateur|Ils croquent près du muret.
-narrateur|Le muret est un peu rêche.
-narrateur|Le jus est sucré.
-maman|Bravo.
-maman|Tu as montré l'abeille.
-enfant-f|On peut la revoir ?
-maman|Un dernier regard.
-narrateur|L'abeille brille encore.
-narrateur|La poule picore plus loin.
-narrateur|La plume ne tourne plus.
-enfant-f|Ce soir, le pain et le miel.
-maman|Oui.
-maman|Avec le petit pot.
-copain|Sur le pain chaud.
-narrateur|Le panier sent déjà le sucré.</t>
+          <t>narrateur|Nina veut prendre le pot, trop vite.
+enfant-f|Je le mets, d'un coup !
+narrateur|Le pot glisse vers le bord.
+enfant-f|Ça tombe !
+copain|Attends.
+narrateur|Aniss recule d'un pas.
+narrateur|Nina avance les mains, trop vite.
+narrateur|Elle regarde les lunettes, trop longtemps.
+narrateur|Un rire revient dans sa bouche.
+copain|Non.
+enfant-f|Oh.
+narrateur|Le pot penche, collant.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe l'abeille, un instant.
+narrateur|Elle écoute le rotin du panier.
+narrateur|Au bord, un éclat de rotin luit.
+enfant-f|Là, sur le bord.
+enfant-f|Tu tiens avec moi ?
+narrateur|Aniss ne dit rien.
+narrateur|Il pose les mains sur le pot.
+copain|Oui.
+narrateur|Ils posent le pot, sans se presser.
+narrateur|L'abeille en bois reste collée.
+enfant-f|Elle est là.
+copain|Derrière.
+papa|Tu l'as montrée, Nina ?
+enfant-f|Oui, papa.
+maman|Le gilet est chaud, Aniss ?
+copain|Un peu.
+narrateur|Le pot glisse dans le panier.
+papa|On passe près du muret ?
+copain|J'y vais.
+narrateur|Nina marche à côté d'Aniss.
+narrateur|Le gilet bleu bouge.
+narrateur|Les lunettes restent sur le nez.
+enfant-f|C'est plus facile.
+papa|Le panier est lourd ?
+enfant-f|Un peu, papa.
+maman|Un rayon passe entre les toiles.
+enfant-f|Il allume le pot.
+narrateur|Ils passent près des prunes.
+enfant-f|Elles sont lisses.
+maman|On va jusqu'au muret ?
+enfant-f|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>pots</t>
         </is>
       </c>
     </row>
@@ -1953,17 +2045,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le miel est dans le panier. L'abeille reste collée sur la caisse. On l'a trouvée. Oui. Vous avez vu l'abeille. La paille sent encore le grain.</t>
+          <t>Ils s'arrêtent près du muret. Maman essuie un peu de sucré. On a vu l'abeille, papa. Tu l'as vue, toi ? Oui, derrière. On est bien, ici. Nina tapote le bord du panier. Il a une trace de rotin. Tu la vois, la trace ? Oui, maman. Le panier est resté, Nina. Oui, avec Aniss. Le panier est resté. Ça sent le pain, un peu tiède. Et les pots, maman. Oui, dans l'air. L'abeille en bois reste collée. Un éclat de rotin tient au bord.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le miel est dans le panier. L'abeille reste collée sur la caisse. On l'a trouvée. Oui. Vous avez vu l'abeille. La paille sent encore le grain.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils s'arrêtent près du muret. Maman essuie un peu de sucré. On a vu l'abeille, papa. Tu l'as vue, toi ? Oui, derrière. On est bien, ici. Nina tapote le bord du panier. Il a une trace de rotin. Tu la vois, la trace ? Oui, maman. Le panier est resté, Nina. Oui, avec Aniss. Le panier est resté. Ça sent le pain, un peu tiède. Et les pots, maman. Oui, dans l'air. L'abeille en bois reste collée. Un &lt;emphasis level="moderate"&gt;éclat de rotin&lt;/emphasis&gt; tient au bord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils s'arrêtent près du muret. Maman essuie un peu de sucré. On a vu l'abeille, papa. Tu l'as vue, toi ? Oui, derrière. On est bien, ici. Nina tapote le bord du panier. Il a une trace de rotin. Tu la vois, la trace ? Oui, maman. Le panier est resté, Nina. Oui, avec Aniss. Le panier est resté. Ça sent le pain, un peu tiède. Et les pots, maman. Oui, dans l'air. L'abeille en bois reste collée. Un &lt;emphasis&gt;éclat de rotin&lt;/emphasis&gt; tient au bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2010,18 +2102,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2030,12 +2122,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2044,17 +2136,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de rotin</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2063,11 +2159,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2076,29 +2172,50 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_au_bord; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le miel est dans le panier.
-narrateur|L'abeille reste collée sur la caisse.
-enfant-f|On l'a trouvée.
-maman|Oui.
-maman|Vous avez vu l'abeille.
-narrateur|La paille sent encore le grain.</t>
+          <t>narrateur|Ils s'arrêtent près du muret.
+narrateur|Maman essuie un peu de sucré.
+enfant-f|On a vu l'abeille, papa.
+papa|Tu l'as vue, toi ?
+enfant-f|Oui, derrière.
+maman|On est bien, ici.
+narrateur|Nina tapote le bord du panier.
+enfant-f|Il a une trace de rotin.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|Le panier est resté, Nina.
+enfant-f|Oui, avec Aniss.
+copain|Le panier est resté.
+narrateur|Ça sent le pain, un peu tiède.
+enfant-f|Et les pots, maman.
+maman|Oui, dans l'air.
+narrateur|L'abeille en bois reste collée.
+narrateur|Un éclat de rotin tient au bord.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>marche</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2204,6 +2321,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>